<commit_message>
add EFO terms to align with new GBD terms
</commit_message>
<xml_diff>
--- a/Data/Second_part_GBD.xlsx
+++ b/Data/Second_part_GBD.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10611"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10102"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rayanaloliet/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jw12513/git/GWAS-GBD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D41CBC3A-3ABA-FC4F-BC02-D433E913CCF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{762869A9-C41E-0F42-B67E-E19305584816}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="500" windowWidth="25300" windowHeight="14600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="298">
   <si>
     <t>GBD term</t>
   </si>
@@ -893,6 +893,27 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Other endocrine, metabolic, blood, and immune disorders</t>
+  </si>
+  <si>
+    <t>Crohn's disease</t>
+  </si>
+  <si>
+    <t>Ulcerative colitis</t>
+  </si>
+  <si>
+    <t>Thyroid diseases</t>
+  </si>
+  <si>
+    <t>EFO:0000384</t>
+  </si>
+  <si>
+    <t>EFO:0000729</t>
+  </si>
+  <si>
+    <t>EFO:1000627</t>
   </si>
 </sst>
 </file>
@@ -916,12 +937,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -936,11 +963,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1245,10 +1273,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N85"/>
+  <dimension ref="A1:N89"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="35.6640625" customWidth="1"/>
+    <col min="1" max="1" width="42.6640625" customWidth="1"/>
     <col min="2" max="9" width="22.33203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1700,7 +1728,7 @@
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
+      <c r="A34" s="2" t="s">
         <v>118</v>
       </c>
       <c r="B34" t="s">
@@ -2341,6 +2369,47 @@
       </c>
       <c r="C85" t="s">
         <v>289</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
+        <v>291</v>
+      </c>
+      <c r="B86" t="s">
+        <v>121</v>
+      </c>
+      <c r="C86" t="s">
+        <v>124</v>
+      </c>
+      <c r="D86" t="s">
+        <v>125</v>
+      </c>
+      <c r="E86" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>292</v>
+      </c>
+      <c r="B87" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>293</v>
+      </c>
+      <c r="B88" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>294</v>
+      </c>
+      <c r="B89" t="s">
+        <v>297</v>
       </c>
     </row>
   </sheetData>

</xml_diff>